<commit_message>
feat(evals): per-stage retrieval attribution + Langfuse scores
Track chunks at three pipeline stages — raw (post-fusion), cutoff
(post-rerank threshold + knee), and final (post-dedup + per-course cap) —
each tallied by RRF source tag (vector_only / bm25_only / overlap) so
counts sum to the stage total. Adds chunk_tokens for context-size analysis.

All 13 metrics emit as Langfuse scores per trace, surfacing as columns in
the dataset-run view next to context_precision / context_recall so runs
of the same dataset are directly comparable when tuning knobs like
retrieve_k or the per-course cap.

Backfill scripts walk every past trace of ragas_20260519_curated20_v2,
parse the existing search / rerank / node.retrieval observations
(chunk_tokens reconstructed from node.retrieval output — no MongoDB
lookup needed), delete the obsolete first-iteration score names, and
post the new schema.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tamu_data/evals/reports/eval_curated20_v2_baseline_20260519_20260519_231827.xlsx
+++ b/tamu_data/evals/reports/eval_curated20_v2_baseline_20260519_20260519_231827.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column Definitions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Per-Query'!$A$1:$AF$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Per-Query'!$A$1:$AG$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -660,6 +660,16 @@
       </c>
       <c r="B20" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mean chunk tokens (backfilled)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2396.6</v>
       </c>
     </row>
   </sheetData>
@@ -673,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF12"/>
+  <dimension ref="A1:AG12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -773,100 +783,105 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>chunk_tokens</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>est_output_tokens</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>citation_pass</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ragas_faithfulness</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ragas_relevancy</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>context_precision</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>context_recall</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>pipeline_ms</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>generator_ms</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>total_ms</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>is_recurrent</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>router_ms</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>retrieval_ms</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>generator_node_ms</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>anchor_ms</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>eval_search_ms</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>schedule_filter_ms</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>merge_ms</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>answer_preview</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>human_judgment</t>
         </is>
@@ -917,46 +932,49 @@
       <c r="L2" s="2" t="n">
         <v>368</v>
       </c>
-      <c r="M2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2" t="n"/>
+      <c r="M2" t="n">
+        <v>245</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n">
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R2" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="S2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="2" t="n">
         <v>5421.2</v>
       </c>
-      <c r="T2" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="2" t="n">
         <v>5421.2</v>
       </c>
-      <c r="V2" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W2" s="2" t="n">
+      <c r="W2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X2" s="2" t="n">
         <v>4480</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="Y2" s="2" t="n">
         <v>476.1</v>
       </c>
-      <c r="Y2" s="2" t="n"/>
       <c r="Z2" s="2" t="n"/>
       <c r="AA2" s="2" t="n"/>
       <c r="AB2" s="2" t="n"/>
       <c r="AC2" s="2" t="n"/>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="n"/>
-      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="n"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="n"/>
+      <c r="AG2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -995,40 +1013,43 @@
       <c r="L3" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="M3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="n"/>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="n">
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="n">
         <v>10334.4</v>
       </c>
-      <c r="T3" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="2" t="n">
         <v>10334.4</v>
       </c>
-      <c r="V3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W3" s="2" t="n">
+      <c r="W3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X3" s="2" t="n">
         <v>2466</v>
       </c>
-      <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="n"/>
       <c r="Z3" s="2" t="n"/>
       <c r="AA3" s="2" t="n"/>
       <c r="AB3" s="2" t="n"/>
       <c r="AC3" s="2" t="n"/>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="n"/>
-      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="n"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="n"/>
+      <c r="AG3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1071,42 +1092,45 @@
       <c r="L4" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" s="2" t="n"/>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n">
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="n">
         <v>2847.5</v>
       </c>
-      <c r="T4" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="2" t="n">
         <v>2847.5</v>
       </c>
-      <c r="V4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W4" s="2" t="n">
+      <c r="W4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X4" s="2" t="n">
         <v>2394</v>
       </c>
-      <c r="X4" s="2" t="n">
+      <c r="Y4" s="2" t="n">
         <v>288.8</v>
       </c>
-      <c r="Y4" s="2" t="n"/>
       <c r="Z4" s="2" t="n"/>
       <c r="AA4" s="2" t="n"/>
       <c r="AB4" s="2" t="n"/>
       <c r="AC4" s="2" t="n"/>
-      <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="n"/>
-      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="n"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="n"/>
+      <c r="AG4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1149,46 +1173,49 @@
       <c r="L5" s="2" t="n">
         <v>566</v>
       </c>
-      <c r="M5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" s="2" t="n"/>
+      <c r="M5" t="n">
+        <v>526</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="2" t="n">
         <v>8770.5</v>
       </c>
-      <c r="T5" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="2" t="n">
         <v>8770.5</v>
       </c>
-      <c r="V5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W5" s="2" t="n">
+      <c r="W5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X5" s="2" t="n">
         <v>7724.1</v>
       </c>
-      <c r="X5" s="2" t="n">
+      <c r="Y5" s="2" t="n">
         <v>588.1</v>
       </c>
-      <c r="Y5" s="2" t="n"/>
       <c r="Z5" s="2" t="n"/>
       <c r="AA5" s="2" t="n"/>
       <c r="AB5" s="2" t="n"/>
       <c r="AC5" s="2" t="n"/>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="n"/>
-      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="n"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="n"/>
+      <c r="AG5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1231,46 +1258,49 @@
       <c r="L6" s="2" t="n">
         <v>1231</v>
       </c>
-      <c r="M6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" s="2" t="n"/>
+      <c r="M6" t="n">
+        <v>1133</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P6" s="2" t="n"/>
-      <c r="Q6" s="2" t="n">
+      <c r="Q6" s="2" t="n"/>
+      <c r="R6" s="2" t="n">
         <v>0.4167</v>
       </c>
-      <c r="R6" s="2" t="n">
+      <c r="S6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S6" s="2" t="n">
+      <c r="T6" s="2" t="n">
         <v>11181.1</v>
       </c>
-      <c r="T6" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="2" t="n">
         <v>11181.1</v>
       </c>
-      <c r="V6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W6" s="2" t="n">
+      <c r="W6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X6" s="2" t="n">
         <v>10383.6</v>
       </c>
-      <c r="X6" s="2" t="n">
+      <c r="Y6" s="2" t="n">
         <v>599.2</v>
       </c>
-      <c r="Y6" s="2" t="n"/>
       <c r="Z6" s="2" t="n"/>
       <c r="AA6" s="2" t="n"/>
       <c r="AB6" s="2" t="n"/>
       <c r="AC6" s="2" t="n"/>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="n"/>
-      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="n"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="n"/>
+      <c r="AG6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1313,46 +1343,49 @@
       <c r="L7" s="2" t="n">
         <v>3424</v>
       </c>
-      <c r="M7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2" t="n"/>
+      <c r="M7" t="n">
+        <v>3411</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="Q7" s="2" t="n"/>
       <c r="R7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="S7" s="2" t="n">
+      <c r="T7" s="2" t="n">
         <v>2579.1</v>
       </c>
-      <c r="T7" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="2" t="n">
         <v>2579.1</v>
       </c>
-      <c r="V7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W7" s="2" t="n">
+      <c r="W7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X7" s="2" t="n">
         <v>1686.5</v>
       </c>
-      <c r="X7" s="2" t="n">
+      <c r="Y7" s="2" t="n">
         <v>556.4</v>
       </c>
-      <c r="Y7" s="2" t="n"/>
       <c r="Z7" s="2" t="n"/>
       <c r="AA7" s="2" t="n"/>
       <c r="AB7" s="2" t="n"/>
       <c r="AC7" s="2" t="n"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="n"/>
-      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="n"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="n"/>
+      <c r="AG7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1395,46 +1428,49 @@
       <c r="L8" s="2" t="n">
         <v>6464</v>
       </c>
-      <c r="M8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" s="2" t="n"/>
+      <c r="M8" t="n">
+        <v>6414</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="n">
         <v>3034.5</v>
       </c>
-      <c r="T8" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="2" t="n">
         <v>3034.5</v>
       </c>
-      <c r="V8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W8" s="2" t="n">
+      <c r="W8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X8" s="2" t="n">
         <v>2238.6</v>
       </c>
-      <c r="X8" s="2" t="n">
+      <c r="Y8" s="2" t="n">
         <v>594.3</v>
       </c>
-      <c r="Y8" s="2" t="n"/>
       <c r="Z8" s="2" t="n"/>
       <c r="AA8" s="2" t="n"/>
       <c r="AB8" s="2" t="n"/>
       <c r="AC8" s="2" t="n"/>
-      <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="n"/>
-      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="n"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="n"/>
+      <c r="AG8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1473,40 +1509,43 @@
       <c r="L9" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="M9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O9" s="2" t="n"/>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
       <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="n">
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="n">
         <v>6880.1</v>
       </c>
-      <c r="T9" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="2" t="n">
         <v>6880.1</v>
       </c>
-      <c r="V9" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W9" s="2" t="n">
+      <c r="W9" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X9" s="2" t="n">
         <v>3315</v>
       </c>
-      <c r="X9" s="2" t="n"/>
       <c r="Y9" s="2" t="n"/>
       <c r="Z9" s="2" t="n"/>
       <c r="AA9" s="2" t="n"/>
       <c r="AB9" s="2" t="n"/>
       <c r="AC9" s="2" t="n"/>
-      <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="n"/>
-      <c r="AF9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="n"/>
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="n"/>
+      <c r="AG9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1549,46 +1588,49 @@
       <c r="L10" s="2" t="n">
         <v>4807</v>
       </c>
-      <c r="M10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O10" s="2" t="n"/>
+      <c r="M10" t="n">
+        <v>4766</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="n">
+      <c r="Q10" s="2" t="n"/>
+      <c r="R10" s="2" t="n">
         <v>0.7133</v>
       </c>
-      <c r="R10" s="2" t="n">
+      <c r="S10" s="2" t="n">
         <v>0.6</v>
       </c>
-      <c r="S10" s="2" t="n">
+      <c r="T10" s="2" t="n">
         <v>3315.8</v>
       </c>
-      <c r="T10" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="2" t="n">
         <v>3315.8</v>
       </c>
-      <c r="V10" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W10" s="2" t="n">
+      <c r="W10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X10" s="2" t="n">
         <v>2419.3</v>
       </c>
-      <c r="X10" s="2" t="n">
+      <c r="Y10" s="2" t="n">
         <v>658</v>
       </c>
-      <c r="Y10" s="2" t="n"/>
       <c r="Z10" s="2" t="n"/>
       <c r="AA10" s="2" t="n"/>
       <c r="AB10" s="2" t="n"/>
       <c r="AC10" s="2" t="n"/>
-      <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="n"/>
-      <c r="AF10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="n"/>
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="n"/>
+      <c r="AG10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1631,46 +1673,49 @@
       <c r="L11" s="2" t="n">
         <v>4385</v>
       </c>
-      <c r="M11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O11" s="2" t="n"/>
+      <c r="M11" t="n">
+        <v>4369</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P11" s="2" t="n"/>
-      <c r="Q11" s="2" t="n">
+      <c r="Q11" s="2" t="n"/>
+      <c r="R11" s="2" t="n">
         <v>0.1036</v>
       </c>
-      <c r="R11" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="n">
         <v>2727.7</v>
       </c>
-      <c r="T11" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="2" t="n">
         <v>2727.7</v>
       </c>
-      <c r="V11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W11" s="2" t="n">
+      <c r="W11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X11" s="2" t="n">
         <v>1980.5</v>
       </c>
-      <c r="X11" s="2" t="n">
+      <c r="Y11" s="2" t="n">
         <v>557.6</v>
       </c>
-      <c r="Y11" s="2" t="n"/>
       <c r="Z11" s="2" t="n"/>
       <c r="AA11" s="2" t="n"/>
       <c r="AB11" s="2" t="n"/>
       <c r="AC11" s="2" t="n"/>
-      <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="n"/>
-      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="n"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="n"/>
+      <c r="AG11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1713,49 +1758,52 @@
       <c r="L12" s="2" t="n">
         <v>5596</v>
       </c>
-      <c r="M12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O12" s="2" t="n"/>
+      <c r="M12" t="n">
+        <v>5499</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="Q12" s="2" t="n"/>
       <c r="R12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
         <v>3928.6</v>
       </c>
-      <c r="T12" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="U12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="2" t="n">
         <v>3928.6</v>
       </c>
-      <c r="V12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="W12" s="2" t="n">
+      <c r="W12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X12" s="2" t="n">
         <v>3150.6</v>
       </c>
-      <c r="X12" s="2" t="n">
+      <c r="Y12" s="2" t="n">
         <v>543.7</v>
       </c>
-      <c r="Y12" s="2" t="n"/>
       <c r="Z12" s="2" t="n"/>
       <c r="AA12" s="2" t="n"/>
       <c r="AB12" s="2" t="n"/>
       <c r="AC12" s="2" t="n"/>
-      <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="n"/>
-      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="n"/>
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="n"/>
+      <c r="AG12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF12"/>
+  <autoFilter ref="A1:AG12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2117,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2652,6 +2700,23 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>chunk_tokens</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Backfilled: estimated tokens in retrieved chunk content only (no query). Computed as est_input_tokens - len(question)//4. Approximation only — the run-time formula floors the combined sum, which can differ from subtracting floored components by at most 1.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>